<commit_message>
feat: Add Med_Norm_When_Present and Med_Norm_All_Recipes to clean87 ingredient statistics
</commit_message>
<xml_diff>
--- a/outputs/pca_v2_noOT_ingredient_statistics_clean87.xlsx
+++ b/outputs/pca_v2_noOT_ingredient_statistics_clean87.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,38 +425,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F226"/>
+  <dimension ref="A1:H226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>CAS</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ingredient</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Frequency</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Recipes_Count</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Avg_Norm_When_Present</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Avg_Norm_All_Recipes</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Med_Norm_When_Present</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Med_Norm_All_Recipes</t>
         </is>
       </c>
     </row>
@@ -471,6 +493,12 @@
       <c r="F2" t="n">
         <v>0.09965499999999999</v>
       </c>
+      <c r="G2" t="n">
+        <v>0.077262</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.077262</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -495,6 +523,12 @@
       <c r="F3" t="n">
         <v>0.033897</v>
       </c>
+      <c r="G3" t="n">
+        <v>0.02468</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.022849</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -519,6 +553,12 @@
       <c r="F4" t="n">
         <v>0.035488</v>
       </c>
+      <c r="G4" t="n">
+        <v>0.028382</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.027825</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -543,6 +583,12 @@
       <c r="F5" t="n">
         <v>0.044638</v>
       </c>
+      <c r="G5" t="n">
+        <v>0.038634</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.036009</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -567,6 +613,12 @@
       <c r="F6" t="n">
         <v>0.076115</v>
       </c>
+      <c r="G6" t="n">
+        <v>0.055078</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.044732</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -591,6 +643,12 @@
       <c r="F7" t="n">
         <v>0.052047</v>
       </c>
+      <c r="G7" t="n">
+        <v>0.051147</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.036469</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -615,6 +673,12 @@
       <c r="F8" t="n">
         <v>0.072281</v>
       </c>
+      <c r="G8" t="n">
+        <v>0.042611</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.020307</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -639,6 +703,12 @@
       <c r="F9" t="n">
         <v>0.014347</v>
       </c>
+      <c r="G9" t="n">
+        <v>0.013165</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.007216</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -663,6 +733,12 @@
       <c r="F10" t="n">
         <v>0.007742</v>
       </c>
+      <c r="G10" t="n">
+        <v>0.004982</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.002161</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -687,6 +763,12 @@
       <c r="F11" t="n">
         <v>0.023567</v>
       </c>
+      <c r="G11" t="n">
+        <v>0.010918</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.005266</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -711,6 +793,12 @@
       <c r="F12" t="n">
         <v>0.024328</v>
       </c>
+      <c r="G12" t="n">
+        <v>0.018231</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.001745</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -735,6 +823,12 @@
       <c r="F13" t="n">
         <v>0.008449999999999999</v>
       </c>
+      <c r="G13" t="n">
+        <v>0.008965000000000001</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.0008899999999999999</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -759,6 +853,12 @@
       <c r="F14" t="n">
         <v>0.015525</v>
       </c>
+      <c r="G14" t="n">
+        <v>0.011142</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4.9e-05</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -783,6 +883,12 @@
       <c r="F15" t="n">
         <v>0.023937</v>
       </c>
+      <c r="G15" t="n">
+        <v>0.031302</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -807,6 +913,12 @@
       <c r="F16" t="n">
         <v>0.027045</v>
       </c>
+      <c r="G16" t="n">
+        <v>0.055357</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -831,6 +943,12 @@
       <c r="F17" t="n">
         <v>0.018491</v>
       </c>
+      <c r="G17" t="n">
+        <v>0.010484</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -855,6 +973,12 @@
       <c r="F18" t="n">
         <v>0.013658</v>
       </c>
+      <c r="G18" t="n">
+        <v>0.024125</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -879,6 +1003,12 @@
       <c r="F19" t="n">
         <v>0.003371</v>
       </c>
+      <c r="G19" t="n">
+        <v>0.007444</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -903,6 +1033,12 @@
       <c r="F20" t="n">
         <v>0.005295</v>
       </c>
+      <c r="G20" t="n">
+        <v>0.006691</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -927,6 +1063,12 @@
       <c r="F21" t="n">
         <v>0.002572</v>
       </c>
+      <c r="G21" t="n">
+        <v>0.006503</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -951,6 +1093,12 @@
       <c r="F22" t="n">
         <v>0.000922</v>
       </c>
+      <c r="G22" t="n">
+        <v>0.00059</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -975,6 +1123,12 @@
       <c r="F23" t="n">
         <v>0.001907</v>
       </c>
+      <c r="G23" t="n">
+        <v>0.00378</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -999,6 +1153,12 @@
       <c r="F24" t="n">
         <v>0.000339</v>
       </c>
+      <c r="G24" t="n">
+        <v>0.0006669999999999999</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1023,6 +1183,12 @@
       <c r="F25" t="n">
         <v>0.001135</v>
       </c>
+      <c r="G25" t="n">
+        <v>0.001164</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1047,6 +1213,12 @@
       <c r="F26" t="n">
         <v>0.003239</v>
       </c>
+      <c r="G26" t="n">
+        <v>0.005706</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1071,6 +1243,12 @@
       <c r="F27" t="n">
         <v>0.001323</v>
       </c>
+      <c r="G27" t="n">
+        <v>0.000458</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1095,6 +1273,12 @@
       <c r="F28" t="n">
         <v>0.001344</v>
       </c>
+      <c r="G28" t="n">
+        <v>0.003489</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1119,6 +1303,12 @@
       <c r="F29" t="n">
         <v>0.000131</v>
       </c>
+      <c r="G29" t="n">
+        <v>4.2e-05</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1143,6 +1333,12 @@
       <c r="F30" t="n">
         <v>0.001012</v>
       </c>
+      <c r="G30" t="n">
+        <v>0.000975</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1167,6 +1363,12 @@
       <c r="F31" t="n">
         <v>0.003291</v>
       </c>
+      <c r="G31" t="n">
+        <v>0.002618</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1191,6 +1393,12 @@
       <c r="F32" t="n">
         <v>0.00141</v>
       </c>
+      <c r="G32" t="n">
+        <v>0.008833000000000001</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1215,6 +1423,12 @@
       <c r="F33" t="n">
         <v>0.003013</v>
       </c>
+      <c r="G33" t="n">
+        <v>0.001023</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1239,6 +1453,12 @@
       <c r="F34" t="n">
         <v>0.00026</v>
       </c>
+      <c r="G34" t="n">
+        <v>0.000733</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1263,6 +1483,12 @@
       <c r="F35" t="n">
         <v>0.000563</v>
       </c>
+      <c r="G35" t="n">
+        <v>0.002591</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1287,6 +1513,12 @@
       <c r="F36" t="n">
         <v>0.004403</v>
       </c>
+      <c r="G36" t="n">
+        <v>0.01788</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1311,6 +1543,12 @@
       <c r="F37" t="n">
         <v>0.000113</v>
       </c>
+      <c r="G37" t="n">
+        <v>0.000648</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1335,6 +1573,12 @@
       <c r="F38" t="n">
         <v>0.000142</v>
       </c>
+      <c r="G38" t="n">
+        <v>0.000423</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1359,6 +1603,12 @@
       <c r="F39" t="n">
         <v>0.000185</v>
       </c>
+      <c r="G39" t="n">
+        <v>0.000777</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1383,6 +1633,12 @@
       <c r="F40" t="n">
         <v>0.001269</v>
       </c>
+      <c r="G40" t="n">
+        <v>0.006874</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1407,6 +1663,12 @@
       <c r="F41" t="n">
         <v>0.003121</v>
       </c>
+      <c r="G41" t="n">
+        <v>0.026445</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1431,6 +1693,12 @@
       <c r="F42" t="n">
         <v>0.00016</v>
       </c>
+      <c r="G42" t="n">
+        <v>0.000703</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1455,6 +1723,12 @@
       <c r="F43" t="n">
         <v>7.4e-05</v>
       </c>
+      <c r="G43" t="n">
+        <v>0.000277</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1479,6 +1753,12 @@
       <c r="F44" t="n">
         <v>0.001138</v>
       </c>
+      <c r="G44" t="n">
+        <v>0.001501</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1503,6 +1783,12 @@
       <c r="F45" t="n">
         <v>0.000211</v>
       </c>
+      <c r="G45" t="n">
+        <v>0.000784</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1527,6 +1813,12 @@
       <c r="F46" t="n">
         <v>0.000246</v>
       </c>
+      <c r="G46" t="n">
+        <v>0.000298</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1551,6 +1843,12 @@
       <c r="F47" t="n">
         <v>0.0001</v>
       </c>
+      <c r="G47" t="n">
+        <v>0.000896</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1575,6 +1873,12 @@
       <c r="F48" t="n">
         <v>0.000435</v>
       </c>
+      <c r="G48" t="n">
+        <v>0.002357</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1599,6 +1903,12 @@
       <c r="F49" t="n">
         <v>0.001121</v>
       </c>
+      <c r="G49" t="n">
+        <v>0.011432</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1623,6 +1933,12 @@
       <c r="F50" t="n">
         <v>6.2e-05</v>
       </c>
+      <c r="G50" t="n">
+        <v>0.000147</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1647,6 +1963,12 @@
       <c r="F51" t="n">
         <v>0.00032</v>
       </c>
+      <c r="G51" t="n">
+        <v>0.002232</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1671,6 +1993,12 @@
       <c r="F52" t="n">
         <v>0.002581</v>
       </c>
+      <c r="G52" t="n">
+        <v>0.016776</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1695,6 +2023,12 @@
       <c r="F53" t="n">
         <v>0.001311</v>
       </c>
+      <c r="G53" t="n">
+        <v>0.006006</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1719,6 +2053,12 @@
       <c r="F54" t="n">
         <v>0.000112</v>
       </c>
+      <c r="G54" t="n">
+        <v>0.001184</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1743,6 +2083,12 @@
       <c r="F55" t="n">
         <v>0.000341</v>
       </c>
+      <c r="G55" t="n">
+        <v>0.000324</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1767,6 +2113,12 @@
       <c r="F56" t="n">
         <v>7.2e-05</v>
       </c>
+      <c r="G56" t="n">
+        <v>0.000687</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1791,6 +2143,12 @@
       <c r="F57" t="n">
         <v>8.1e-05</v>
       </c>
+      <c r="G57" t="n">
+        <v>7.8e-05</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1815,6 +2173,12 @@
       <c r="F58" t="n">
         <v>2e-06</v>
       </c>
+      <c r="G58" t="n">
+        <v>2.4e-05</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1839,6 +2203,12 @@
       <c r="F59" t="n">
         <v>0.000242</v>
       </c>
+      <c r="G59" t="n">
+        <v>0.003437</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1863,6 +2233,12 @@
       <c r="F60" t="n">
         <v>3.1e-05</v>
       </c>
+      <c r="G60" t="n">
+        <v>0.000727</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1887,6 +2263,12 @@
       <c r="F61" t="n">
         <v>0.0006310000000000001</v>
       </c>
+      <c r="G61" t="n">
+        <v>0.001259</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1911,6 +2293,12 @@
       <c r="F62" t="n">
         <v>0.000288</v>
       </c>
+      <c r="G62" t="n">
+        <v>0.003756</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1935,6 +2323,12 @@
       <c r="F63" t="n">
         <v>7e-06</v>
       </c>
+      <c r="G63" t="n">
+        <v>7.9e-05</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1959,6 +2353,12 @@
       <c r="F64" t="n">
         <v>2.2e-05</v>
       </c>
+      <c r="G64" t="n">
+        <v>0.00049</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1983,6 +2383,12 @@
       <c r="F65" t="n">
         <v>0.000351</v>
       </c>
+      <c r="G65" t="n">
+        <v>0.006065</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2007,6 +2413,12 @@
       <c r="F66" t="n">
         <v>1.9e-05</v>
       </c>
+      <c r="G66" t="n">
+        <v>0.000382</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2031,6 +2443,12 @@
       <c r="F67" t="n">
         <v>1e-05</v>
       </c>
+      <c r="G67" t="n">
+        <v>0.000207</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2055,6 +2473,12 @@
       <c r="F68" t="n">
         <v>3.8e-05</v>
       </c>
+      <c r="G68" t="n">
+        <v>0.000556</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2079,6 +2503,12 @@
       <c r="F69" t="n">
         <v>3.6e-05</v>
       </c>
+      <c r="G69" t="n">
+        <v>0.000569</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2103,6 +2533,12 @@
       <c r="F70" t="n">
         <v>4.1e-05</v>
       </c>
+      <c r="G70" t="n">
+        <v>0.000178</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2127,6 +2563,12 @@
       <c r="F71" t="n">
         <v>0.000199</v>
       </c>
+      <c r="G71" t="n">
+        <v>0.003541</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2151,6 +2593,12 @@
       <c r="F72" t="n">
         <v>0.000291</v>
       </c>
+      <c r="G72" t="n">
+        <v>0.007674</v>
+      </c>
+      <c r="H72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2175,6 +2623,12 @@
       <c r="F73" t="n">
         <v>6e-05</v>
       </c>
+      <c r="G73" t="n">
+        <v>0.000917</v>
+      </c>
+      <c r="H73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2199,6 +2653,12 @@
       <c r="F74" t="n">
         <v>9e-06</v>
       </c>
+      <c r="G74" t="n">
+        <v>0.000274</v>
+      </c>
+      <c r="H74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2223,6 +2683,12 @@
       <c r="F75" t="n">
         <v>4.1e-05</v>
       </c>
+      <c r="G75" t="n">
+        <v>0.00045</v>
+      </c>
+      <c r="H75" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2247,6 +2713,12 @@
       <c r="F76" t="n">
         <v>1e-06</v>
       </c>
+      <c r="G76" t="n">
+        <v>5.2e-05</v>
+      </c>
+      <c r="H76" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2271,6 +2743,12 @@
       <c r="F77" t="n">
         <v>1e-06</v>
       </c>
+      <c r="G77" t="n">
+        <v>2.1e-05</v>
+      </c>
+      <c r="H77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2295,6 +2773,12 @@
       <c r="F78" t="n">
         <v>0.001671</v>
       </c>
+      <c r="G78" t="n">
+        <v>5e-06</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2319,6 +2803,12 @@
       <c r="F79" t="n">
         <v>1.9e-05</v>
       </c>
+      <c r="G79" t="n">
+        <v>0.000325</v>
+      </c>
+      <c r="H79" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2343,6 +2833,12 @@
       <c r="F80" t="n">
         <v>0.0009120000000000001</v>
       </c>
+      <c r="G80" t="n">
+        <v>0.039651</v>
+      </c>
+      <c r="H80" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2367,6 +2863,12 @@
       <c r="F81" t="n">
         <v>0.000325</v>
       </c>
+      <c r="G81" t="n">
+        <v>0.014158</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2391,6 +2893,12 @@
       <c r="F82" t="n">
         <v>2.2e-05</v>
       </c>
+      <c r="G82" t="n">
+        <v>0.000942</v>
+      </c>
+      <c r="H82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2415,6 +2923,12 @@
       <c r="F83" t="n">
         <v>6e-06</v>
       </c>
+      <c r="G83" t="n">
+        <v>0.000256</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2439,6 +2953,12 @@
       <c r="F84" t="n">
         <v>0.000137</v>
       </c>
+      <c r="G84" t="n">
+        <v>0.00596</v>
+      </c>
+      <c r="H84" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2463,6 +2983,12 @@
       <c r="F85" t="n">
         <v>0.000152</v>
       </c>
+      <c r="G85" t="n">
+        <v>0.006593</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2487,6 +3013,12 @@
       <c r="F86" t="n">
         <v>0.000285</v>
       </c>
+      <c r="G86" t="n">
+        <v>0.012392</v>
+      </c>
+      <c r="H86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2511,6 +3043,12 @@
       <c r="F87" t="n">
         <v>1e-05</v>
       </c>
+      <c r="G87" t="n">
+        <v>0.000414</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2535,6 +3073,12 @@
       <c r="F88" t="n">
         <v>0.000187</v>
       </c>
+      <c r="G88" t="n">
+        <v>0.008149</v>
+      </c>
+      <c r="H88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2559,6 +3103,12 @@
       <c r="F89" t="n">
         <v>2.5e-05</v>
       </c>
+      <c r="G89" t="n">
+        <v>0.001083</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2583,6 +3133,12 @@
       <c r="F90" t="n">
         <v>7.4e-05</v>
       </c>
+      <c r="G90" t="n">
+        <v>0.003208</v>
+      </c>
+      <c r="H90" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2607,6 +3163,12 @@
       <c r="F91" t="n">
         <v>0.000491</v>
       </c>
+      <c r="G91" t="n">
+        <v>0.021368</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2631,6 +3193,12 @@
       <c r="F92" t="n">
         <v>5.7e-05</v>
       </c>
+      <c r="G92" t="n">
+        <v>0.002483</v>
+      </c>
+      <c r="H92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2655,6 +3223,12 @@
       <c r="F93" t="n">
         <v>8e-06</v>
       </c>
+      <c r="G93" t="n">
+        <v>0.000354</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2679,6 +3253,12 @@
       <c r="F94" t="n">
         <v>1.5e-05</v>
       </c>
+      <c r="G94" t="n">
+        <v>0.000664</v>
+      </c>
+      <c r="H94" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2703,6 +3283,12 @@
       <c r="F95" t="n">
         <v>1.9e-05</v>
       </c>
+      <c r="G95" t="n">
+        <v>0.000837</v>
+      </c>
+      <c r="H95" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2727,6 +3313,12 @@
       <c r="F96" t="n">
         <v>9.399999999999999e-05</v>
       </c>
+      <c r="G96" t="n">
+        <v>0.00409</v>
+      </c>
+      <c r="H96" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2751,6 +3343,12 @@
       <c r="F97" t="n">
         <v>1.8e-05</v>
       </c>
+      <c r="G97" t="n">
+        <v>0.000781</v>
+      </c>
+      <c r="H97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2775,6 +3373,12 @@
       <c r="F98" t="n">
         <v>3.2e-05</v>
       </c>
+      <c r="G98" t="n">
+        <v>0.001379</v>
+      </c>
+      <c r="H98" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2799,6 +3403,12 @@
       <c r="F99" t="n">
         <v>0.000229</v>
       </c>
+      <c r="G99" t="n">
+        <v>0.009965</v>
+      </c>
+      <c r="H99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2823,6 +3433,12 @@
       <c r="F100" t="n">
         <v>0</v>
       </c>
+      <c r="G100" t="n">
+        <v>2e-05</v>
+      </c>
+      <c r="H100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2847,6 +3463,12 @@
       <c r="F101" t="n">
         <v>1.7e-05</v>
       </c>
+      <c r="G101" t="n">
+        <v>0.000759</v>
+      </c>
+      <c r="H101" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2871,6 +3493,12 @@
       <c r="F102" t="n">
         <v>4e-06</v>
       </c>
+      <c r="G102" t="n">
+        <v>0.000345</v>
+      </c>
+      <c r="H102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2895,6 +3523,12 @@
       <c r="F103" t="n">
         <v>1.5e-05</v>
       </c>
+      <c r="G103" t="n">
+        <v>0.001321</v>
+      </c>
+      <c r="H103" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2919,6 +3553,12 @@
       <c r="F104" t="n">
         <v>1.3e-05</v>
       </c>
+      <c r="G104" t="n">
+        <v>0.00114</v>
+      </c>
+      <c r="H104" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2943,6 +3583,12 @@
       <c r="F105" t="n">
         <v>0.000252</v>
       </c>
+      <c r="G105" t="n">
+        <v>0.02195</v>
+      </c>
+      <c r="H105" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2967,6 +3613,12 @@
       <c r="F106" t="n">
         <v>5e-06</v>
       </c>
+      <c r="G106" t="n">
+        <v>0.00044</v>
+      </c>
+      <c r="H106" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2991,6 +3643,12 @@
       <c r="F107" t="n">
         <v>0.000174</v>
       </c>
+      <c r="G107" t="n">
+        <v>0.015147</v>
+      </c>
+      <c r="H107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3015,6 +3673,12 @@
       <c r="F108" t="n">
         <v>3e-06</v>
       </c>
+      <c r="G108" t="n">
+        <v>0.000246</v>
+      </c>
+      <c r="H108" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3039,6 +3703,12 @@
       <c r="F109" t="n">
         <v>1.5e-05</v>
       </c>
+      <c r="G109" t="n">
+        <v>0.001275</v>
+      </c>
+      <c r="H109" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3063,6 +3733,12 @@
       <c r="F110" t="n">
         <v>3.8e-05</v>
       </c>
+      <c r="G110" t="n">
+        <v>0.003281</v>
+      </c>
+      <c r="H110" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3087,6 +3763,12 @@
       <c r="F111" t="n">
         <v>3e-06</v>
       </c>
+      <c r="G111" t="n">
+        <v>0.000298</v>
+      </c>
+      <c r="H111" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3111,6 +3793,12 @@
       <c r="F112" t="n">
         <v>1.2e-05</v>
       </c>
+      <c r="G112" t="n">
+        <v>0.001024</v>
+      </c>
+      <c r="H112" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3135,6 +3823,12 @@
       <c r="F113" t="n">
         <v>2.2e-05</v>
       </c>
+      <c r="G113" t="n">
+        <v>0.001896</v>
+      </c>
+      <c r="H113" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3159,6 +3853,12 @@
       <c r="F114" t="n">
         <v>3e-06</v>
       </c>
+      <c r="G114" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H114" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3183,6 +3883,12 @@
       <c r="F115" t="n">
         <v>1e-06</v>
       </c>
+      <c r="G115" t="n">
+        <v>9.899999999999999e-05</v>
+      </c>
+      <c r="H115" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3207,6 +3913,12 @@
       <c r="F116" t="n">
         <v>0.001097</v>
       </c>
+      <c r="G116" t="n">
+        <v>0.09547700000000001</v>
+      </c>
+      <c r="H116" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3231,6 +3943,12 @@
       <c r="F117" t="n">
         <v>5.3e-05</v>
       </c>
+      <c r="G117" t="n">
+        <v>0.004605</v>
+      </c>
+      <c r="H117" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3255,6 +3973,12 @@
       <c r="F118" t="n">
         <v>2.6e-05</v>
       </c>
+      <c r="G118" t="n">
+        <v>0.002269</v>
+      </c>
+      <c r="H118" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3279,6 +4003,12 @@
       <c r="F119" t="n">
         <v>3e-06</v>
       </c>
+      <c r="G119" t="n">
+        <v>0.000227</v>
+      </c>
+      <c r="H119" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3303,6 +4033,12 @@
       <c r="F120" t="n">
         <v>1e-06</v>
       </c>
+      <c r="G120" t="n">
+        <v>8.899999999999999e-05</v>
+      </c>
+      <c r="H120" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3327,6 +4063,12 @@
       <c r="F121" t="n">
         <v>1.5e-05</v>
       </c>
+      <c r="G121" t="n">
+        <v>0.001278</v>
+      </c>
+      <c r="H121" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3351,6 +4093,12 @@
       <c r="F122" t="n">
         <v>3e-06</v>
       </c>
+      <c r="G122" t="n">
+        <v>0.000264</v>
+      </c>
+      <c r="H122" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3375,6 +4123,12 @@
       <c r="F123" t="n">
         <v>2.7e-05</v>
       </c>
+      <c r="G123" t="n">
+        <v>0.002344</v>
+      </c>
+      <c r="H123" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3399,6 +4153,12 @@
       <c r="F124" t="n">
         <v>3.1e-05</v>
       </c>
+      <c r="G124" t="n">
+        <v>0.002675</v>
+      </c>
+      <c r="H124" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3423,6 +4183,12 @@
       <c r="F125" t="n">
         <v>1e-06</v>
       </c>
+      <c r="G125" t="n">
+        <v>0.000119</v>
+      </c>
+      <c r="H125" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3447,6 +4213,12 @@
       <c r="F126" t="n">
         <v>0</v>
       </c>
+      <c r="G126" t="n">
+        <v>2.9e-05</v>
+      </c>
+      <c r="H126" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3471,6 +4243,12 @@
       <c r="F127" t="n">
         <v>2.9e-05</v>
       </c>
+      <c r="G127" t="n">
+        <v>0.002549</v>
+      </c>
+      <c r="H127" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3495,6 +4273,12 @@
       <c r="F128" t="n">
         <v>9.2e-05</v>
       </c>
+      <c r="G128" t="n">
+        <v>0.008009</v>
+      </c>
+      <c r="H128" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3519,6 +4303,12 @@
       <c r="F129" t="n">
         <v>1e-06</v>
       </c>
+      <c r="G129" t="n">
+        <v>8.2e-05</v>
+      </c>
+      <c r="H129" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -3543,6 +4333,12 @@
       <c r="F130" t="n">
         <v>0.000859</v>
       </c>
+      <c r="G130" t="n">
+        <v>0.074752</v>
+      </c>
+      <c r="H130" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -3567,6 +4363,12 @@
       <c r="F131" t="n">
         <v>3.2e-05</v>
       </c>
+      <c r="G131" t="n">
+        <v>0.002789</v>
+      </c>
+      <c r="H131" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -3591,6 +4393,12 @@
       <c r="F132" t="n">
         <v>5e-06</v>
       </c>
+      <c r="G132" t="n">
+        <v>0.000426</v>
+      </c>
+      <c r="H132" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -3615,6 +4423,12 @@
       <c r="F133" t="n">
         <v>0.000109</v>
       </c>
+      <c r="G133" t="n">
+        <v>0.009450999999999999</v>
+      </c>
+      <c r="H133" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -3639,6 +4453,12 @@
       <c r="F134" t="n">
         <v>0</v>
       </c>
+      <c r="G134" t="n">
+        <v>8e-06</v>
+      </c>
+      <c r="H134" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -3663,6 +4483,12 @@
       <c r="F135" t="n">
         <v>1e-06</v>
       </c>
+      <c r="G135" t="n">
+        <v>8.500000000000001e-05</v>
+      </c>
+      <c r="H135" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -3687,6 +4513,12 @@
       <c r="F136" t="n">
         <v>0</v>
       </c>
+      <c r="G136" t="n">
+        <v>3.7e-05</v>
+      </c>
+      <c r="H136" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -3709,6 +4541,10 @@
       <c r="F137" t="n">
         <v>0</v>
       </c>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -3731,6 +4567,10 @@
       <c r="F138" t="n">
         <v>0</v>
       </c>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -3753,6 +4593,10 @@
       <c r="F139" t="n">
         <v>0</v>
       </c>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -3775,6 +4619,10 @@
       <c r="F140" t="n">
         <v>0</v>
       </c>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -3797,6 +4645,10 @@
       <c r="F141" t="n">
         <v>0</v>
       </c>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -3819,6 +4671,10 @@
       <c r="F142" t="n">
         <v>0</v>
       </c>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3841,6 +4697,10 @@
       <c r="F143" t="n">
         <v>0</v>
       </c>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3863,6 +4723,10 @@
       <c r="F144" t="n">
         <v>0</v>
       </c>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3885,6 +4749,10 @@
       <c r="F145" t="n">
         <v>0</v>
       </c>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3907,6 +4775,10 @@
       <c r="F146" t="n">
         <v>0</v>
       </c>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3929,6 +4801,10 @@
       <c r="F147" t="n">
         <v>0</v>
       </c>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -3951,6 +4827,10 @@
       <c r="F148" t="n">
         <v>0</v>
       </c>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -3973,6 +4853,10 @@
       <c r="F149" t="n">
         <v>0</v>
       </c>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -3995,6 +4879,10 @@
       <c r="F150" t="n">
         <v>0</v>
       </c>
+      <c r="G150" t="inlineStr"/>
+      <c r="H150" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -4017,6 +4905,10 @@
       <c r="F151" t="n">
         <v>0</v>
       </c>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -4039,6 +4931,10 @@
       <c r="F152" t="n">
         <v>0</v>
       </c>
+      <c r="G152" t="inlineStr"/>
+      <c r="H152" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -4061,6 +4957,10 @@
       <c r="F153" t="n">
         <v>0</v>
       </c>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -4083,6 +4983,10 @@
       <c r="F154" t="n">
         <v>0</v>
       </c>
+      <c r="G154" t="inlineStr"/>
+      <c r="H154" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -4105,6 +5009,10 @@
       <c r="F155" t="n">
         <v>0</v>
       </c>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -4127,6 +5035,10 @@
       <c r="F156" t="n">
         <v>0</v>
       </c>
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -4149,6 +5061,10 @@
       <c r="F157" t="n">
         <v>0</v>
       </c>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -4171,6 +5087,10 @@
       <c r="F158" t="n">
         <v>0</v>
       </c>
+      <c r="G158" t="inlineStr"/>
+      <c r="H158" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -4193,6 +5113,10 @@
       <c r="F159" t="n">
         <v>0</v>
       </c>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -4215,6 +5139,10 @@
       <c r="F160" t="n">
         <v>0</v>
       </c>
+      <c r="G160" t="inlineStr"/>
+      <c r="H160" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -4237,6 +5165,10 @@
       <c r="F161" t="n">
         <v>0</v>
       </c>
+      <c r="G161" t="inlineStr"/>
+      <c r="H161" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -4259,6 +5191,10 @@
       <c r="F162" t="n">
         <v>0</v>
       </c>
+      <c r="G162" t="inlineStr"/>
+      <c r="H162" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -4281,6 +5217,10 @@
       <c r="F163" t="n">
         <v>0</v>
       </c>
+      <c r="G163" t="inlineStr"/>
+      <c r="H163" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -4303,6 +5243,10 @@
       <c r="F164" t="n">
         <v>0</v>
       </c>
+      <c r="G164" t="inlineStr"/>
+      <c r="H164" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -4325,6 +5269,10 @@
       <c r="F165" t="n">
         <v>0</v>
       </c>
+      <c r="G165" t="inlineStr"/>
+      <c r="H165" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -4347,6 +5295,10 @@
       <c r="F166" t="n">
         <v>0</v>
       </c>
+      <c r="G166" t="inlineStr"/>
+      <c r="H166" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -4369,6 +5321,10 @@
       <c r="F167" t="n">
         <v>0</v>
       </c>
+      <c r="G167" t="inlineStr"/>
+      <c r="H167" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -4391,6 +5347,10 @@
       <c r="F168" t="n">
         <v>0</v>
       </c>
+      <c r="G168" t="inlineStr"/>
+      <c r="H168" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -4413,6 +5373,10 @@
       <c r="F169" t="n">
         <v>0</v>
       </c>
+      <c r="G169" t="inlineStr"/>
+      <c r="H169" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -4435,6 +5399,10 @@
       <c r="F170" t="n">
         <v>0</v>
       </c>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -4457,6 +5425,10 @@
       <c r="F171" t="n">
         <v>0</v>
       </c>
+      <c r="G171" t="inlineStr"/>
+      <c r="H171" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -4479,6 +5451,10 @@
       <c r="F172" t="n">
         <v>0</v>
       </c>
+      <c r="G172" t="inlineStr"/>
+      <c r="H172" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -4501,6 +5477,10 @@
       <c r="F173" t="n">
         <v>0</v>
       </c>
+      <c r="G173" t="inlineStr"/>
+      <c r="H173" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -4523,6 +5503,10 @@
       <c r="F174" t="n">
         <v>0</v>
       </c>
+      <c r="G174" t="inlineStr"/>
+      <c r="H174" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -4545,6 +5529,10 @@
       <c r="F175" t="n">
         <v>0</v>
       </c>
+      <c r="G175" t="inlineStr"/>
+      <c r="H175" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -4567,6 +5555,10 @@
       <c r="F176" t="n">
         <v>0</v>
       </c>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -4589,6 +5581,10 @@
       <c r="F177" t="n">
         <v>0</v>
       </c>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -4611,6 +5607,10 @@
       <c r="F178" t="n">
         <v>0</v>
       </c>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -4633,6 +5633,10 @@
       <c r="F179" t="n">
         <v>0</v>
       </c>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -4655,6 +5659,10 @@
       <c r="F180" t="n">
         <v>0</v>
       </c>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -4677,6 +5685,10 @@
       <c r="F181" t="n">
         <v>0</v>
       </c>
+      <c r="G181" t="inlineStr"/>
+      <c r="H181" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -4699,6 +5711,10 @@
       <c r="F182" t="n">
         <v>0</v>
       </c>
+      <c r="G182" t="inlineStr"/>
+      <c r="H182" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -4721,6 +5737,10 @@
       <c r="F183" t="n">
         <v>0</v>
       </c>
+      <c r="G183" t="inlineStr"/>
+      <c r="H183" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -4743,6 +5763,10 @@
       <c r="F184" t="n">
         <v>0</v>
       </c>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -4765,6 +5789,10 @@
       <c r="F185" t="n">
         <v>0</v>
       </c>
+      <c r="G185" t="inlineStr"/>
+      <c r="H185" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -4787,6 +5815,10 @@
       <c r="F186" t="n">
         <v>0</v>
       </c>
+      <c r="G186" t="inlineStr"/>
+      <c r="H186" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -4809,6 +5841,10 @@
       <c r="F187" t="n">
         <v>0</v>
       </c>
+      <c r="G187" t="inlineStr"/>
+      <c r="H187" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -4831,6 +5867,10 @@
       <c r="F188" t="n">
         <v>0</v>
       </c>
+      <c r="G188" t="inlineStr"/>
+      <c r="H188" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -4853,6 +5893,10 @@
       <c r="F189" t="n">
         <v>0</v>
       </c>
+      <c r="G189" t="inlineStr"/>
+      <c r="H189" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -4875,6 +5919,10 @@
       <c r="F190" t="n">
         <v>0</v>
       </c>
+      <c r="G190" t="inlineStr"/>
+      <c r="H190" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -4897,6 +5945,10 @@
       <c r="F191" t="n">
         <v>0</v>
       </c>
+      <c r="G191" t="inlineStr"/>
+      <c r="H191" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -4919,6 +5971,10 @@
       <c r="F192" t="n">
         <v>0</v>
       </c>
+      <c r="G192" t="inlineStr"/>
+      <c r="H192" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -4941,6 +5997,10 @@
       <c r="F193" t="n">
         <v>0</v>
       </c>
+      <c r="G193" t="inlineStr"/>
+      <c r="H193" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -4963,6 +6023,10 @@
       <c r="F194" t="n">
         <v>0</v>
       </c>
+      <c r="G194" t="inlineStr"/>
+      <c r="H194" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -4985,6 +6049,10 @@
       <c r="F195" t="n">
         <v>0</v>
       </c>
+      <c r="G195" t="inlineStr"/>
+      <c r="H195" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -5007,6 +6075,10 @@
       <c r="F196" t="n">
         <v>0</v>
       </c>
+      <c r="G196" t="inlineStr"/>
+      <c r="H196" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -5029,6 +6101,10 @@
       <c r="F197" t="n">
         <v>0</v>
       </c>
+      <c r="G197" t="inlineStr"/>
+      <c r="H197" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -5051,6 +6127,10 @@
       <c r="F198" t="n">
         <v>0</v>
       </c>
+      <c r="G198" t="inlineStr"/>
+      <c r="H198" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -5073,6 +6153,10 @@
       <c r="F199" t="n">
         <v>0</v>
       </c>
+      <c r="G199" t="inlineStr"/>
+      <c r="H199" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -5095,6 +6179,10 @@
       <c r="F200" t="n">
         <v>0</v>
       </c>
+      <c r="G200" t="inlineStr"/>
+      <c r="H200" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -5117,6 +6205,10 @@
       <c r="F201" t="n">
         <v>0</v>
       </c>
+      <c r="G201" t="inlineStr"/>
+      <c r="H201" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -5139,6 +6231,10 @@
       <c r="F202" t="n">
         <v>0</v>
       </c>
+      <c r="G202" t="inlineStr"/>
+      <c r="H202" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -5161,6 +6257,10 @@
       <c r="F203" t="n">
         <v>0</v>
       </c>
+      <c r="G203" t="inlineStr"/>
+      <c r="H203" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -5183,6 +6283,10 @@
       <c r="F204" t="n">
         <v>0</v>
       </c>
+      <c r="G204" t="inlineStr"/>
+      <c r="H204" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -5205,6 +6309,10 @@
       <c r="F205" t="n">
         <v>0</v>
       </c>
+      <c r="G205" t="inlineStr"/>
+      <c r="H205" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -5227,6 +6335,10 @@
       <c r="F206" t="n">
         <v>0</v>
       </c>
+      <c r="G206" t="inlineStr"/>
+      <c r="H206" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -5249,6 +6361,10 @@
       <c r="F207" t="n">
         <v>0</v>
       </c>
+      <c r="G207" t="inlineStr"/>
+      <c r="H207" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -5271,6 +6387,10 @@
       <c r="F208" t="n">
         <v>0</v>
       </c>
+      <c r="G208" t="inlineStr"/>
+      <c r="H208" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -5293,6 +6413,10 @@
       <c r="F209" t="n">
         <v>0</v>
       </c>
+      <c r="G209" t="inlineStr"/>
+      <c r="H209" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -5315,6 +6439,10 @@
       <c r="F210" t="n">
         <v>0</v>
       </c>
+      <c r="G210" t="inlineStr"/>
+      <c r="H210" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -5337,6 +6465,10 @@
       <c r="F211" t="n">
         <v>0</v>
       </c>
+      <c r="G211" t="inlineStr"/>
+      <c r="H211" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -5359,6 +6491,10 @@
       <c r="F212" t="n">
         <v>0</v>
       </c>
+      <c r="G212" t="inlineStr"/>
+      <c r="H212" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -5381,6 +6517,10 @@
       <c r="F213" t="n">
         <v>0</v>
       </c>
+      <c r="G213" t="inlineStr"/>
+      <c r="H213" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -5403,6 +6543,10 @@
       <c r="F214" t="n">
         <v>0</v>
       </c>
+      <c r="G214" t="inlineStr"/>
+      <c r="H214" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -5425,6 +6569,10 @@
       <c r="F215" t="n">
         <v>0</v>
       </c>
+      <c r="G215" t="inlineStr"/>
+      <c r="H215" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -5447,6 +6595,10 @@
       <c r="F216" t="n">
         <v>0</v>
       </c>
+      <c r="G216" t="inlineStr"/>
+      <c r="H216" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -5469,6 +6621,10 @@
       <c r="F217" t="n">
         <v>0</v>
       </c>
+      <c r="G217" t="inlineStr"/>
+      <c r="H217" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -5491,6 +6647,10 @@
       <c r="F218" t="n">
         <v>0</v>
       </c>
+      <c r="G218" t="inlineStr"/>
+      <c r="H218" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -5513,6 +6673,10 @@
       <c r="F219" t="n">
         <v>0</v>
       </c>
+      <c r="G219" t="inlineStr"/>
+      <c r="H219" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -5535,6 +6699,10 @@
       <c r="F220" t="n">
         <v>0</v>
       </c>
+      <c r="G220" t="inlineStr"/>
+      <c r="H220" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -5557,6 +6725,10 @@
       <c r="F221" t="n">
         <v>0</v>
       </c>
+      <c r="G221" t="inlineStr"/>
+      <c r="H221" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -5579,6 +6751,10 @@
       <c r="F222" t="n">
         <v>0</v>
       </c>
+      <c r="G222" t="inlineStr"/>
+      <c r="H222" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -5601,6 +6777,10 @@
       <c r="F223" t="n">
         <v>0</v>
       </c>
+      <c r="G223" t="inlineStr"/>
+      <c r="H223" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -5623,6 +6803,10 @@
       <c r="F224" t="n">
         <v>0</v>
       </c>
+      <c r="G224" t="inlineStr"/>
+      <c r="H224" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -5645,6 +6829,10 @@
       <c r="F225" t="n">
         <v>0</v>
       </c>
+      <c r="G225" t="inlineStr"/>
+      <c r="H225" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -5665,6 +6853,10 @@
       </c>
       <c r="E226" t="inlineStr"/>
       <c r="F226" t="n">
+        <v>0</v>
+      </c>
+      <c r="G226" t="inlineStr"/>
+      <c r="H226" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>